<commit_message>
update data package at: 2026-08-27T14:21:00
</commit_message>
<xml_diff>
--- a/data/BASE_DETALHAMENTO_OBRAS.xlsx
+++ b/data/BASE_DETALHAMENTO_OBRAS.xlsx
@@ -6692,8 +6692,10 @@
           <t>INICIANDO</t>
         </is>
       </c>
-      <c r="L97" t="n">
-        <v>207</v>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>UNIDADE</t>
+        </is>
       </c>
       <c r="M97" t="n">
         <v>1</v>
@@ -8558,8 +8560,10 @@
           <t>PARALISADO</t>
         </is>
       </c>
-      <c r="L126" t="n">
-        <v>130</v>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>METRO QUADRADO</t>
+        </is>
       </c>
       <c r="M126" t="n">
         <v>5000</v>
@@ -9438,8 +9442,10 @@
           <t>EXECUÇÃO</t>
         </is>
       </c>
-      <c r="L140" t="n">
-        <v>207</v>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>UNIDADE</t>
+        </is>
       </c>
       <c r="M140" t="n">
         <v>1</v>
@@ -9574,8 +9580,10 @@
           <t>EXECUÇÃO</t>
         </is>
       </c>
-      <c r="L142" t="n">
-        <v>207</v>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>UNIDADE</t>
+        </is>
       </c>
       <c r="M142" t="n">
         <v>1</v>
@@ -9644,8 +9652,10 @@
           <t>EXECUÇÃO</t>
         </is>
       </c>
-      <c r="L143" t="n">
-        <v>207</v>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>UNIDADE</t>
+        </is>
       </c>
       <c r="M143" t="n">
         <v>1</v>
@@ -9912,8 +9922,10 @@
           <t>EXECUÇÃO</t>
         </is>
       </c>
-      <c r="L147" t="n">
-        <v>207</v>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>UNIDADE</t>
+        </is>
       </c>
       <c r="M147" t="n">
         <v>1</v>
@@ -9982,8 +9994,10 @@
           <t>EXECUÇÃO</t>
         </is>
       </c>
-      <c r="L148" t="n">
-        <v>207</v>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>UNIDADE</t>
+        </is>
       </c>
       <c r="M148" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
update data package at: 2026-08-27T14:25:31
</commit_message>
<xml_diff>
--- a/data/BASE_DETALHAMENTO_OBRAS.xlsx
+++ b/data/BASE_DETALHAMENTO_OBRAS.xlsx
@@ -560,7 +560,9 @@
       <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="inlineStr"/>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
@@ -624,7 +626,9 @@
       <c r="G3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="inlineStr"/>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
@@ -688,7 +692,9 @@
       <c r="G4" t="n">
         <v>0</v>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="n">
+        <v>3</v>
+      </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
@@ -752,7 +758,9 @@
       <c r="G5" t="n">
         <v>1</v>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="n">
+        <v>4</v>
+      </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
@@ -816,7 +824,9 @@
       <c r="G6" t="n">
         <v>1</v>
       </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="H6" t="n">
+        <v>5</v>
+      </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
@@ -880,7 +890,9 @@
       <c r="G7" t="n">
         <v>1</v>
       </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="n">
+        <v>6</v>
+      </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
@@ -944,7 +956,9 @@
       <c r="G8" t="n">
         <v>1</v>
       </c>
-      <c r="H8" t="inlineStr"/>
+      <c r="H8" t="n">
+        <v>7</v>
+      </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
@@ -1008,7 +1022,9 @@
       <c r="G9" t="n">
         <v>1</v>
       </c>
-      <c r="H9" t="inlineStr"/>
+      <c r="H9" t="n">
+        <v>8</v>
+      </c>
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
@@ -1072,7 +1088,9 @@
       <c r="G10" t="n">
         <v>1</v>
       </c>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>9</v>
+      </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
@@ -1136,7 +1154,9 @@
       <c r="G11" t="n">
         <v>1</v>
       </c>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>10</v>
+      </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
@@ -1200,7 +1220,9 @@
       <c r="G12" t="n">
         <v>1</v>
       </c>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>11</v>
+      </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
@@ -1264,7 +1286,9 @@
       <c r="G13" t="n">
         <v>1</v>
       </c>
-      <c r="H13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>12</v>
+      </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
@@ -1328,7 +1352,9 @@
       <c r="G14" t="n">
         <v>1</v>
       </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>13</v>
+      </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
@@ -1392,7 +1418,9 @@
       <c r="G15" t="n">
         <v>1</v>
       </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>14</v>
+      </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
@@ -1456,7 +1484,9 @@
       <c r="G16" t="n">
         <v>1</v>
       </c>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>15</v>
+      </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
         <is>
@@ -1520,7 +1550,9 @@
       <c r="G17" t="n">
         <v>1</v>
       </c>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>16</v>
+      </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr">
         <is>
@@ -1584,7 +1616,9 @@
       <c r="G18" t="n">
         <v>1</v>
       </c>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>17</v>
+      </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr">
         <is>
@@ -1648,7 +1682,9 @@
       <c r="G19" t="n">
         <v>1</v>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>18</v>
+      </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr">
         <is>
@@ -1712,7 +1748,9 @@
       <c r="G20" t="n">
         <v>1</v>
       </c>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>19</v>
+      </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
@@ -1776,7 +1814,9 @@
       <c r="G21" t="n">
         <v>1</v>
       </c>
-      <c r="H21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>20</v>
+      </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
@@ -1840,7 +1880,9 @@
       <c r="G22" t="n">
         <v>1</v>
       </c>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>21</v>
+      </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
         <is>
@@ -1904,7 +1946,9 @@
       <c r="G23" t="n">
         <v>1</v>
       </c>
-      <c r="H23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>22</v>
+      </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
@@ -1968,7 +2012,9 @@
       <c r="G24" t="n">
         <v>1</v>
       </c>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>23</v>
+      </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr">
         <is>
@@ -2032,7 +2078,9 @@
       <c r="G25" t="n">
         <v>1</v>
       </c>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>24</v>
+      </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
@@ -2096,7 +2144,9 @@
       <c r="G26" t="n">
         <v>1</v>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>25</v>
+      </c>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr">
         <is>
@@ -2160,7 +2210,9 @@
       <c r="G27" t="n">
         <v>1</v>
       </c>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="n">
+        <v>26</v>
+      </c>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr">
         <is>
@@ -2224,7 +2276,9 @@
       <c r="G28" t="n">
         <v>1</v>
       </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>27</v>
+      </c>
       <c r="I28" t="inlineStr"/>
       <c r="J28" t="inlineStr">
         <is>
@@ -2288,7 +2342,9 @@
       <c r="G29" t="n">
         <v>1</v>
       </c>
-      <c r="H29" t="inlineStr"/>
+      <c r="H29" t="n">
+        <v>28</v>
+      </c>
       <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr">
         <is>
@@ -2352,7 +2408,9 @@
       <c r="G30" t="n">
         <v>1</v>
       </c>
-      <c r="H30" t="inlineStr"/>
+      <c r="H30" t="n">
+        <v>29</v>
+      </c>
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
@@ -2416,7 +2474,9 @@
       <c r="G31" t="n">
         <v>1</v>
       </c>
-      <c r="H31" t="inlineStr"/>
+      <c r="H31" t="n">
+        <v>30</v>
+      </c>
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
@@ -2480,7 +2540,9 @@
       <c r="G32" t="n">
         <v>1</v>
       </c>
-      <c r="H32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>31</v>
+      </c>
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
@@ -2544,7 +2606,9 @@
       <c r="G33" t="n">
         <v>1</v>
       </c>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="n">
+        <v>32</v>
+      </c>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
@@ -2608,7 +2672,9 @@
       <c r="G34" t="n">
         <v>1</v>
       </c>
-      <c r="H34" t="inlineStr"/>
+      <c r="H34" t="n">
+        <v>33</v>
+      </c>
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
@@ -2672,7 +2738,9 @@
       <c r="G35" t="n">
         <v>1</v>
       </c>
-      <c r="H35" t="inlineStr"/>
+      <c r="H35" t="n">
+        <v>34</v>
+      </c>
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
@@ -2736,7 +2804,9 @@
       <c r="G36" t="n">
         <v>1</v>
       </c>
-      <c r="H36" t="inlineStr"/>
+      <c r="H36" t="n">
+        <v>35</v>
+      </c>
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
@@ -2800,7 +2870,9 @@
       <c r="G37" t="n">
         <v>1</v>
       </c>
-      <c r="H37" t="inlineStr"/>
+      <c r="H37" t="n">
+        <v>36</v>
+      </c>
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
@@ -2864,7 +2936,9 @@
       <c r="G38" t="n">
         <v>1</v>
       </c>
-      <c r="H38" t="inlineStr"/>
+      <c r="H38" t="n">
+        <v>37</v>
+      </c>
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
@@ -2928,7 +3002,9 @@
       <c r="G39" t="n">
         <v>1</v>
       </c>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="n">
+        <v>38</v>
+      </c>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
@@ -2992,7 +3068,9 @@
       <c r="G40" t="n">
         <v>1</v>
       </c>
-      <c r="H40" t="inlineStr"/>
+      <c r="H40" t="n">
+        <v>39</v>
+      </c>
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
@@ -3056,7 +3134,9 @@
       <c r="G41" t="n">
         <v>1</v>
       </c>
-      <c r="H41" t="inlineStr"/>
+      <c r="H41" t="n">
+        <v>40</v>
+      </c>
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
@@ -3120,7 +3200,9 @@
       <c r="G42" t="n">
         <v>1</v>
       </c>
-      <c r="H42" t="inlineStr"/>
+      <c r="H42" t="n">
+        <v>41</v>
+      </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
@@ -3184,7 +3266,9 @@
       <c r="G43" t="n">
         <v>1</v>
       </c>
-      <c r="H43" t="inlineStr"/>
+      <c r="H43" t="n">
+        <v>42</v>
+      </c>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
@@ -3248,7 +3332,9 @@
       <c r="G44" t="n">
         <v>1</v>
       </c>
-      <c r="H44" t="inlineStr"/>
+      <c r="H44" t="n">
+        <v>43</v>
+      </c>
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
@@ -3312,7 +3398,9 @@
       <c r="G45" t="n">
         <v>1</v>
       </c>
-      <c r="H45" t="inlineStr"/>
+      <c r="H45" t="n">
+        <v>44</v>
+      </c>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
@@ -3376,7 +3464,9 @@
       <c r="G46" t="n">
         <v>1</v>
       </c>
-      <c r="H46" t="inlineStr"/>
+      <c r="H46" t="n">
+        <v>45</v>
+      </c>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
@@ -3440,7 +3530,9 @@
       <c r="G47" t="n">
         <v>1</v>
       </c>
-      <c r="H47" t="inlineStr"/>
+      <c r="H47" t="n">
+        <v>46</v>
+      </c>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
@@ -3504,7 +3596,9 @@
       <c r="G48" t="n">
         <v>1</v>
       </c>
-      <c r="H48" t="inlineStr"/>
+      <c r="H48" t="n">
+        <v>47</v>
+      </c>
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
@@ -3568,7 +3662,9 @@
       <c r="G49" t="n">
         <v>1</v>
       </c>
-      <c r="H49" t="inlineStr"/>
+      <c r="H49" t="n">
+        <v>48</v>
+      </c>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
@@ -3632,7 +3728,9 @@
       <c r="G50" t="n">
         <v>1</v>
       </c>
-      <c r="H50" t="inlineStr"/>
+      <c r="H50" t="n">
+        <v>49</v>
+      </c>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
@@ -3696,7 +3794,9 @@
       <c r="G51" t="n">
         <v>1</v>
       </c>
-      <c r="H51" t="inlineStr"/>
+      <c r="H51" t="n">
+        <v>50</v>
+      </c>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
@@ -3760,7 +3860,9 @@
       <c r="G52" t="n">
         <v>1</v>
       </c>
-      <c r="H52" t="inlineStr"/>
+      <c r="H52" t="n">
+        <v>51</v>
+      </c>
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr">
         <is>
@@ -3824,7 +3926,9 @@
       <c r="G53" t="n">
         <v>1</v>
       </c>
-      <c r="H53" t="inlineStr"/>
+      <c r="H53" t="n">
+        <v>52</v>
+      </c>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr">
         <is>
@@ -3888,7 +3992,9 @@
       <c r="G54" t="n">
         <v>1</v>
       </c>
-      <c r="H54" t="inlineStr"/>
+      <c r="H54" t="n">
+        <v>53</v>
+      </c>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr">
         <is>
@@ -3952,7 +4058,9 @@
       <c r="G55" t="n">
         <v>1</v>
       </c>
-      <c r="H55" t="inlineStr"/>
+      <c r="H55" t="n">
+        <v>54</v>
+      </c>
       <c r="I55" t="inlineStr"/>
       <c r="J55" t="inlineStr">
         <is>
@@ -4016,7 +4124,9 @@
       <c r="G56" t="n">
         <v>1</v>
       </c>
-      <c r="H56" t="inlineStr"/>
+      <c r="H56" t="n">
+        <v>55</v>
+      </c>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr">
         <is>
@@ -4080,7 +4190,9 @@
       <c r="G57" t="n">
         <v>1</v>
       </c>
-      <c r="H57" t="inlineStr"/>
+      <c r="H57" t="n">
+        <v>56</v>
+      </c>
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr">
         <is>
@@ -4144,7 +4256,9 @@
       <c r="G58" t="n">
         <v>1</v>
       </c>
-      <c r="H58" t="inlineStr"/>
+      <c r="H58" t="n">
+        <v>57</v>
+      </c>
       <c r="I58" t="inlineStr"/>
       <c r="J58" t="inlineStr">
         <is>
@@ -4208,7 +4322,9 @@
       <c r="G59" t="n">
         <v>1</v>
       </c>
-      <c r="H59" t="inlineStr"/>
+      <c r="H59" t="n">
+        <v>58</v>
+      </c>
       <c r="I59" t="inlineStr"/>
       <c r="J59" t="inlineStr">
         <is>
@@ -4272,7 +4388,9 @@
       <c r="G60" t="n">
         <v>1</v>
       </c>
-      <c r="H60" t="inlineStr"/>
+      <c r="H60" t="n">
+        <v>59</v>
+      </c>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr">
         <is>
@@ -4336,7 +4454,9 @@
       <c r="G61" t="n">
         <v>1</v>
       </c>
-      <c r="H61" t="inlineStr"/>
+      <c r="H61" t="n">
+        <v>60</v>
+      </c>
       <c r="I61" t="inlineStr"/>
       <c r="J61" t="inlineStr">
         <is>
@@ -4400,7 +4520,9 @@
       <c r="G62" t="n">
         <v>1</v>
       </c>
-      <c r="H62" t="inlineStr"/>
+      <c r="H62" t="n">
+        <v>61</v>
+      </c>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr">
         <is>
@@ -4464,7 +4586,9 @@
       <c r="G63" t="n">
         <v>1</v>
       </c>
-      <c r="H63" t="inlineStr"/>
+      <c r="H63" t="n">
+        <v>62</v>
+      </c>
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr">
         <is>
@@ -4528,7 +4652,9 @@
       <c r="G64" t="n">
         <v>1</v>
       </c>
-      <c r="H64" t="inlineStr"/>
+      <c r="H64" t="n">
+        <v>63</v>
+      </c>
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr">
         <is>
@@ -4592,7 +4718,9 @@
       <c r="G65" t="n">
         <v>0</v>
       </c>
-      <c r="H65" t="inlineStr"/>
+      <c r="H65" t="n">
+        <v>64</v>
+      </c>
       <c r="I65" t="n">
         <v>12404</v>
       </c>
@@ -4658,7 +4786,9 @@
       <c r="G66" t="n">
         <v>0</v>
       </c>
-      <c r="H66" t="inlineStr"/>
+      <c r="H66" t="n">
+        <v>65</v>
+      </c>
       <c r="I66" t="n">
         <v>12780</v>
       </c>
@@ -4724,7 +4854,9 @@
       <c r="G67" t="n">
         <v>0</v>
       </c>
-      <c r="H67" t="inlineStr"/>
+      <c r="H67" t="n">
+        <v>66</v>
+      </c>
       <c r="I67" t="n">
         <v>10397</v>
       </c>
@@ -4790,7 +4922,9 @@
       <c r="G68" t="n">
         <v>0</v>
       </c>
-      <c r="H68" t="inlineStr"/>
+      <c r="H68" t="n">
+        <v>67</v>
+      </c>
       <c r="I68" t="n">
         <v>12850</v>
       </c>
@@ -4856,7 +4990,9 @@
       <c r="G69" t="n">
         <v>0</v>
       </c>
-      <c r="H69" t="inlineStr"/>
+      <c r="H69" t="n">
+        <v>68</v>
+      </c>
       <c r="I69" t="n">
         <v>12634</v>
       </c>
@@ -4922,7 +5058,9 @@
       <c r="G70" t="n">
         <v>0</v>
       </c>
-      <c r="H70" t="inlineStr"/>
+      <c r="H70" t="n">
+        <v>69</v>
+      </c>
       <c r="I70" t="n">
         <v>12785</v>
       </c>
@@ -4988,7 +5126,9 @@
       <c r="G71" t="n">
         <v>0</v>
       </c>
-      <c r="H71" t="inlineStr"/>
+      <c r="H71" t="n">
+        <v>70</v>
+      </c>
       <c r="I71" t="n">
         <v>12824</v>
       </c>
@@ -5054,7 +5194,9 @@
       <c r="G72" t="n">
         <v>0</v>
       </c>
-      <c r="H72" t="inlineStr"/>
+      <c r="H72" t="n">
+        <v>71</v>
+      </c>
       <c r="I72" t="n">
         <v>4716</v>
       </c>
@@ -5120,7 +5262,9 @@
       <c r="G73" t="n">
         <v>0</v>
       </c>
-      <c r="H73" t="inlineStr"/>
+      <c r="H73" t="n">
+        <v>72</v>
+      </c>
       <c r="I73" t="n">
         <v>11140</v>
       </c>
@@ -5186,7 +5330,9 @@
       <c r="G74" t="n">
         <v>0</v>
       </c>
-      <c r="H74" t="inlineStr"/>
+      <c r="H74" t="n">
+        <v>73</v>
+      </c>
       <c r="I74" t="n">
         <v>12510</v>
       </c>
@@ -5252,7 +5398,9 @@
       <c r="G75" t="n">
         <v>0</v>
       </c>
-      <c r="H75" t="inlineStr"/>
+      <c r="H75" t="n">
+        <v>74</v>
+      </c>
       <c r="I75" t="n">
         <v>12453</v>
       </c>
@@ -5318,7 +5466,9 @@
       <c r="G76" t="n">
         <v>0</v>
       </c>
-      <c r="H76" t="inlineStr"/>
+      <c r="H76" t="n">
+        <v>75</v>
+      </c>
       <c r="I76" t="n">
         <v>12454</v>
       </c>
@@ -5384,7 +5534,9 @@
       <c r="G77" t="n">
         <v>0</v>
       </c>
-      <c r="H77" t="inlineStr"/>
+      <c r="H77" t="n">
+        <v>76</v>
+      </c>
       <c r="I77" t="n">
         <v>11521</v>
       </c>
@@ -5450,7 +5602,9 @@
       <c r="G78" t="n">
         <v>0</v>
       </c>
-      <c r="H78" t="inlineStr"/>
+      <c r="H78" t="n">
+        <v>77</v>
+      </c>
       <c r="I78" t="n">
         <v>11519</v>
       </c>
@@ -5516,7 +5670,9 @@
       <c r="G79" t="n">
         <v>0</v>
       </c>
-      <c r="H79" t="inlineStr"/>
+      <c r="H79" t="n">
+        <v>78</v>
+      </c>
       <c r="I79" t="n">
         <v>11512</v>
       </c>
@@ -5582,7 +5738,9 @@
       <c r="G80" t="n">
         <v>0</v>
       </c>
-      <c r="H80" t="inlineStr"/>
+      <c r="H80" t="n">
+        <v>79</v>
+      </c>
       <c r="I80" t="n">
         <v>11514</v>
       </c>
@@ -5648,7 +5806,9 @@
       <c r="G81" t="n">
         <v>0</v>
       </c>
-      <c r="H81" t="inlineStr"/>
+      <c r="H81" t="n">
+        <v>80</v>
+      </c>
       <c r="I81" t="n">
         <v>11511</v>
       </c>
@@ -5714,7 +5874,9 @@
       <c r="G82" t="n">
         <v>0</v>
       </c>
-      <c r="H82" t="inlineStr"/>
+      <c r="H82" t="n">
+        <v>81</v>
+      </c>
       <c r="I82" t="n">
         <v>11520</v>
       </c>
@@ -5780,7 +5942,9 @@
       <c r="G83" t="n">
         <v>0</v>
       </c>
-      <c r="H83" t="inlineStr"/>
+      <c r="H83" t="n">
+        <v>82</v>
+      </c>
       <c r="I83" t="n">
         <v>11513</v>
       </c>
@@ -5846,7 +6010,9 @@
       <c r="G84" t="n">
         <v>0</v>
       </c>
-      <c r="H84" t="inlineStr"/>
+      <c r="H84" t="n">
+        <v>83</v>
+      </c>
       <c r="I84" t="n">
         <v>11977</v>
       </c>
@@ -5912,7 +6078,9 @@
       <c r="G85" t="n">
         <v>1</v>
       </c>
-      <c r="H85" t="inlineStr"/>
+      <c r="H85" t="n">
+        <v>84</v>
+      </c>
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr">
         <is>
@@ -5976,7 +6144,9 @@
       <c r="G86" t="n">
         <v>1</v>
       </c>
-      <c r="H86" t="inlineStr"/>
+      <c r="H86" t="n">
+        <v>85</v>
+      </c>
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr">
         <is>
@@ -6040,7 +6210,9 @@
       <c r="G87" t="n">
         <v>1</v>
       </c>
-      <c r="H87" t="inlineStr"/>
+      <c r="H87" t="n">
+        <v>86</v>
+      </c>
       <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr">
         <is>
@@ -6104,7 +6276,9 @@
       <c r="G88" t="n">
         <v>1</v>
       </c>
-      <c r="H88" t="inlineStr"/>
+      <c r="H88" t="n">
+        <v>87</v>
+      </c>
       <c r="I88" t="inlineStr"/>
       <c r="J88" t="inlineStr">
         <is>
@@ -6168,7 +6342,9 @@
       <c r="G89" t="n">
         <v>1</v>
       </c>
-      <c r="H89" t="inlineStr"/>
+      <c r="H89" t="n">
+        <v>88</v>
+      </c>
       <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr">
         <is>
@@ -6232,7 +6408,9 @@
       <c r="G90" t="n">
         <v>1</v>
       </c>
-      <c r="H90" t="inlineStr"/>
+      <c r="H90" t="n">
+        <v>89</v>
+      </c>
       <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr">
         <is>
@@ -6296,7 +6474,9 @@
       <c r="G91" t="n">
         <v>0</v>
       </c>
-      <c r="H91" t="inlineStr"/>
+      <c r="H91" t="n">
+        <v>90</v>
+      </c>
       <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr">
         <is>
@@ -6360,7 +6540,9 @@
       <c r="G92" t="n">
         <v>0</v>
       </c>
-      <c r="H92" t="inlineStr"/>
+      <c r="H92" t="n">
+        <v>91</v>
+      </c>
       <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr">
         <is>
@@ -6424,7 +6606,9 @@
       <c r="G93" t="n">
         <v>0</v>
       </c>
-      <c r="H93" t="inlineStr"/>
+      <c r="H93" t="n">
+        <v>92</v>
+      </c>
       <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr">
         <is>
@@ -6488,7 +6672,9 @@
       <c r="G94" t="n">
         <v>0</v>
       </c>
-      <c r="H94" t="inlineStr"/>
+      <c r="H94" t="n">
+        <v>93</v>
+      </c>
       <c r="I94" t="inlineStr"/>
       <c r="J94" t="inlineStr">
         <is>
@@ -6552,7 +6738,9 @@
       <c r="G95" t="n">
         <v>0</v>
       </c>
-      <c r="H95" t="inlineStr"/>
+      <c r="H95" t="n">
+        <v>94</v>
+      </c>
       <c r="I95" t="inlineStr"/>
       <c r="J95" t="inlineStr">
         <is>
@@ -6616,7 +6804,9 @@
       <c r="G96" t="n">
         <v>0</v>
       </c>
-      <c r="H96" t="inlineStr"/>
+      <c r="H96" t="n">
+        <v>95</v>
+      </c>
       <c r="I96" t="inlineStr"/>
       <c r="J96" t="inlineStr">
         <is>
@@ -6680,7 +6870,9 @@
       <c r="G97" t="n">
         <v>0</v>
       </c>
-      <c r="H97" t="inlineStr"/>
+      <c r="H97" t="n">
+        <v>96</v>
+      </c>
       <c r="I97" t="inlineStr"/>
       <c r="J97" t="inlineStr">
         <is>
@@ -6750,7 +6942,9 @@
       <c r="G98" t="n">
         <v>0</v>
       </c>
-      <c r="H98" t="inlineStr"/>
+      <c r="H98" t="n">
+        <v>97</v>
+      </c>
       <c r="I98" t="inlineStr"/>
       <c r="J98" t="inlineStr">
         <is>
@@ -6814,7 +7008,9 @@
       <c r="G99" t="n">
         <v>0</v>
       </c>
-      <c r="H99" t="inlineStr"/>
+      <c r="H99" t="n">
+        <v>98</v>
+      </c>
       <c r="I99" t="inlineStr"/>
       <c r="J99" t="inlineStr">
         <is>
@@ -6878,7 +7074,9 @@
       <c r="G100" t="n">
         <v>0</v>
       </c>
-      <c r="H100" t="inlineStr"/>
+      <c r="H100" t="n">
+        <v>99</v>
+      </c>
       <c r="I100" t="inlineStr"/>
       <c r="J100" t="inlineStr">
         <is>
@@ -6942,7 +7140,9 @@
       <c r="G101" t="n">
         <v>0</v>
       </c>
-      <c r="H101" t="inlineStr"/>
+      <c r="H101" t="n">
+        <v>100</v>
+      </c>
       <c r="I101" t="n">
         <v>12871</v>
       </c>
@@ -7008,7 +7208,9 @@
       <c r="G102" t="n">
         <v>0</v>
       </c>
-      <c r="H102" t="inlineStr"/>
+      <c r="H102" t="n">
+        <v>101</v>
+      </c>
       <c r="I102" t="n">
         <v>9999</v>
       </c>
@@ -7074,7 +7276,9 @@
       <c r="G103" t="n">
         <v>0</v>
       </c>
-      <c r="H103" t="inlineStr"/>
+      <c r="H103" t="n">
+        <v>102</v>
+      </c>
       <c r="I103" t="n">
         <v>12690</v>
       </c>
@@ -7140,7 +7344,9 @@
       <c r="G104" t="n">
         <v>0</v>
       </c>
-      <c r="H104" t="inlineStr"/>
+      <c r="H104" t="n">
+        <v>103</v>
+      </c>
       <c r="I104" t="inlineStr"/>
       <c r="J104" t="inlineStr">
         <is>
@@ -7204,7 +7410,9 @@
       <c r="G105" t="n">
         <v>0</v>
       </c>
-      <c r="H105" t="inlineStr"/>
+      <c r="H105" t="n">
+        <v>104</v>
+      </c>
       <c r="I105" t="inlineStr"/>
       <c r="J105" t="inlineStr">
         <is>
@@ -7268,7 +7476,9 @@
       <c r="G106" t="n">
         <v>0</v>
       </c>
-      <c r="H106" t="inlineStr"/>
+      <c r="H106" t="n">
+        <v>105</v>
+      </c>
       <c r="I106" t="inlineStr"/>
       <c r="J106" t="inlineStr">
         <is>
@@ -7332,7 +7542,9 @@
       <c r="G107" t="n">
         <v>0</v>
       </c>
-      <c r="H107" t="inlineStr"/>
+      <c r="H107" t="n">
+        <v>106</v>
+      </c>
       <c r="I107" t="inlineStr"/>
       <c r="J107" t="inlineStr">
         <is>
@@ -7396,7 +7608,9 @@
       <c r="G108" t="n">
         <v>0</v>
       </c>
-      <c r="H108" t="inlineStr"/>
+      <c r="H108" t="n">
+        <v>107</v>
+      </c>
       <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr">
         <is>
@@ -7460,7 +7674,9 @@
       <c r="G109" t="n">
         <v>0</v>
       </c>
-      <c r="H109" t="inlineStr"/>
+      <c r="H109" t="n">
+        <v>108</v>
+      </c>
       <c r="I109" t="inlineStr"/>
       <c r="J109" t="inlineStr">
         <is>
@@ -7524,7 +7740,9 @@
       <c r="G110" t="n">
         <v>0</v>
       </c>
-      <c r="H110" t="inlineStr"/>
+      <c r="H110" t="n">
+        <v>109</v>
+      </c>
       <c r="I110" t="inlineStr"/>
       <c r="J110" t="inlineStr">
         <is>
@@ -7588,7 +7806,9 @@
       <c r="G111" t="n">
         <v>0</v>
       </c>
-      <c r="H111" t="inlineStr"/>
+      <c r="H111" t="n">
+        <v>110</v>
+      </c>
       <c r="I111" t="inlineStr"/>
       <c r="J111" t="inlineStr">
         <is>
@@ -7652,7 +7872,9 @@
       <c r="G112" t="n">
         <v>0</v>
       </c>
-      <c r="H112" t="inlineStr"/>
+      <c r="H112" t="n">
+        <v>111</v>
+      </c>
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr">
         <is>
@@ -7716,7 +7938,9 @@
       <c r="G113" t="n">
         <v>0</v>
       </c>
-      <c r="H113" t="inlineStr"/>
+      <c r="H113" t="n">
+        <v>112</v>
+      </c>
       <c r="I113" t="inlineStr"/>
       <c r="J113" t="inlineStr">
         <is>
@@ -7780,7 +8004,9 @@
       <c r="G114" t="n">
         <v>0</v>
       </c>
-      <c r="H114" t="inlineStr"/>
+      <c r="H114" t="n">
+        <v>113</v>
+      </c>
       <c r="I114" t="inlineStr"/>
       <c r="J114" t="inlineStr">
         <is>
@@ -7844,7 +8070,9 @@
       <c r="G115" t="n">
         <v>0</v>
       </c>
-      <c r="H115" t="inlineStr"/>
+      <c r="H115" t="n">
+        <v>114</v>
+      </c>
       <c r="I115" t="inlineStr"/>
       <c r="J115" t="inlineStr">
         <is>
@@ -7908,7 +8136,9 @@
       <c r="G116" t="n">
         <v>0</v>
       </c>
-      <c r="H116" t="inlineStr"/>
+      <c r="H116" t="n">
+        <v>115</v>
+      </c>
       <c r="I116" t="inlineStr"/>
       <c r="J116" t="inlineStr">
         <is>
@@ -7972,7 +8202,9 @@
       <c r="G117" t="n">
         <v>0</v>
       </c>
-      <c r="H117" t="inlineStr"/>
+      <c r="H117" t="n">
+        <v>116</v>
+      </c>
       <c r="I117" t="inlineStr"/>
       <c r="J117" t="inlineStr">
         <is>
@@ -8036,7 +8268,9 @@
       <c r="G118" t="n">
         <v>0</v>
       </c>
-      <c r="H118" t="inlineStr"/>
+      <c r="H118" t="n">
+        <v>117</v>
+      </c>
       <c r="I118" t="inlineStr"/>
       <c r="J118" t="inlineStr">
         <is>
@@ -8100,7 +8334,9 @@
       <c r="G119" t="n">
         <v>0</v>
       </c>
-      <c r="H119" t="inlineStr"/>
+      <c r="H119" t="n">
+        <v>118</v>
+      </c>
       <c r="I119" t="inlineStr"/>
       <c r="J119" t="inlineStr">
         <is>
@@ -8164,7 +8400,9 @@
       <c r="G120" t="n">
         <v>0</v>
       </c>
-      <c r="H120" t="inlineStr"/>
+      <c r="H120" t="n">
+        <v>119</v>
+      </c>
       <c r="I120" t="inlineStr"/>
       <c r="J120" t="inlineStr">
         <is>
@@ -8228,7 +8466,9 @@
       <c r="G121" t="n">
         <v>0</v>
       </c>
-      <c r="H121" t="inlineStr"/>
+      <c r="H121" t="n">
+        <v>120</v>
+      </c>
       <c r="I121" t="inlineStr"/>
       <c r="J121" t="inlineStr">
         <is>
@@ -8292,7 +8532,9 @@
       <c r="G122" t="n">
         <v>0</v>
       </c>
-      <c r="H122" t="inlineStr"/>
+      <c r="H122" t="n">
+        <v>121</v>
+      </c>
       <c r="I122" t="inlineStr"/>
       <c r="J122" t="inlineStr">
         <is>
@@ -8356,7 +8598,9 @@
       <c r="G123" t="n">
         <v>0</v>
       </c>
-      <c r="H123" t="inlineStr"/>
+      <c r="H123" t="n">
+        <v>122</v>
+      </c>
       <c r="I123" t="inlineStr"/>
       <c r="J123" t="inlineStr">
         <is>
@@ -8420,7 +8664,9 @@
       <c r="G124" t="n">
         <v>0</v>
       </c>
-      <c r="H124" t="inlineStr"/>
+      <c r="H124" t="n">
+        <v>123</v>
+      </c>
       <c r="I124" t="inlineStr"/>
       <c r="J124" t="inlineStr">
         <is>
@@ -8484,7 +8730,9 @@
       <c r="G125" t="n">
         <v>0</v>
       </c>
-      <c r="H125" t="inlineStr"/>
+      <c r="H125" t="n">
+        <v>124</v>
+      </c>
       <c r="I125" t="inlineStr"/>
       <c r="J125" t="inlineStr">
         <is>
@@ -8548,7 +8796,9 @@
       <c r="G126" t="n">
         <v>0</v>
       </c>
-      <c r="H126" t="inlineStr"/>
+      <c r="H126" t="n">
+        <v>125</v>
+      </c>
       <c r="I126" t="inlineStr"/>
       <c r="J126" t="inlineStr">
         <is>
@@ -8618,7 +8868,9 @@
       <c r="G127" t="n">
         <v>0</v>
       </c>
-      <c r="H127" t="inlineStr"/>
+      <c r="H127" t="n">
+        <v>126</v>
+      </c>
       <c r="I127" t="inlineStr"/>
       <c r="J127" t="inlineStr">
         <is>
@@ -8682,7 +8934,9 @@
       <c r="G128" t="n">
         <v>0</v>
       </c>
-      <c r="H128" t="inlineStr"/>
+      <c r="H128" t="n">
+        <v>127</v>
+      </c>
       <c r="I128" t="inlineStr"/>
       <c r="J128" t="inlineStr">
         <is>
@@ -8746,7 +9000,9 @@
       <c r="G129" t="n">
         <v>0</v>
       </c>
-      <c r="H129" t="inlineStr"/>
+      <c r="H129" t="n">
+        <v>128</v>
+      </c>
       <c r="I129" t="n">
         <v>11877</v>
       </c>
@@ -8812,7 +9068,9 @@
       <c r="G130" t="n">
         <v>0</v>
       </c>
-      <c r="H130" t="inlineStr"/>
+      <c r="H130" t="n">
+        <v>129</v>
+      </c>
       <c r="I130" t="inlineStr"/>
       <c r="J130" t="inlineStr">
         <is>
@@ -8864,7 +9122,9 @@
       <c r="G131" t="n">
         <v>0</v>
       </c>
-      <c r="H131" t="inlineStr"/>
+      <c r="H131" t="n">
+        <v>130</v>
+      </c>
       <c r="I131" t="inlineStr"/>
       <c r="J131" t="inlineStr">
         <is>
@@ -8916,7 +9176,9 @@
       <c r="G132" t="n">
         <v>0</v>
       </c>
-      <c r="H132" t="inlineStr"/>
+      <c r="H132" t="n">
+        <v>131</v>
+      </c>
       <c r="I132" t="inlineStr"/>
       <c r="J132" t="inlineStr">
         <is>
@@ -8980,7 +9242,9 @@
       <c r="G133" t="n">
         <v>0</v>
       </c>
-      <c r="H133" t="inlineStr"/>
+      <c r="H133" t="n">
+        <v>132</v>
+      </c>
       <c r="I133" t="inlineStr"/>
       <c r="J133" t="inlineStr">
         <is>
@@ -9044,7 +9308,9 @@
       <c r="G134" t="n">
         <v>0</v>
       </c>
-      <c r="H134" t="inlineStr"/>
+      <c r="H134" t="n">
+        <v>133</v>
+      </c>
       <c r="I134" t="inlineStr"/>
       <c r="J134" t="inlineStr">
         <is>
@@ -9108,7 +9374,9 @@
       <c r="G135" t="n">
         <v>0</v>
       </c>
-      <c r="H135" t="inlineStr"/>
+      <c r="H135" t="n">
+        <v>134</v>
+      </c>
       <c r="I135" t="inlineStr"/>
       <c r="J135" t="inlineStr">
         <is>
@@ -9172,7 +9440,9 @@
       <c r="G136" t="n">
         <v>0</v>
       </c>
-      <c r="H136" t="inlineStr"/>
+      <c r="H136" t="n">
+        <v>135</v>
+      </c>
       <c r="I136" t="inlineStr"/>
       <c r="J136" t="inlineStr">
         <is>
@@ -9236,7 +9506,9 @@
       <c r="G137" t="n">
         <v>0</v>
       </c>
-      <c r="H137" t="inlineStr"/>
+      <c r="H137" t="n">
+        <v>136</v>
+      </c>
       <c r="I137" t="inlineStr"/>
       <c r="J137" t="inlineStr">
         <is>
@@ -9300,7 +9572,9 @@
       <c r="G138" t="n">
         <v>0</v>
       </c>
-      <c r="H138" t="inlineStr"/>
+      <c r="H138" t="n">
+        <v>137</v>
+      </c>
       <c r="I138" t="inlineStr"/>
       <c r="J138" t="inlineStr">
         <is>
@@ -9364,7 +9638,9 @@
       <c r="G139" t="n">
         <v>0</v>
       </c>
-      <c r="H139" t="inlineStr"/>
+      <c r="H139" t="n">
+        <v>138</v>
+      </c>
       <c r="I139" t="inlineStr"/>
       <c r="J139" t="inlineStr">
         <is>
@@ -9428,7 +9704,9 @@
       <c r="G140" t="n">
         <v>0</v>
       </c>
-      <c r="H140" t="inlineStr"/>
+      <c r="H140" t="n">
+        <v>139</v>
+      </c>
       <c r="I140" t="n">
         <v>12054</v>
       </c>
@@ -9500,7 +9778,9 @@
       <c r="G141" t="n">
         <v>0</v>
       </c>
-      <c r="H141" t="inlineStr"/>
+      <c r="H141" t="n">
+        <v>140</v>
+      </c>
       <c r="I141" t="n">
         <v>12702</v>
       </c>
@@ -9566,7 +9846,9 @@
       <c r="G142" t="n">
         <v>0</v>
       </c>
-      <c r="H142" t="inlineStr"/>
+      <c r="H142" t="n">
+        <v>141</v>
+      </c>
       <c r="I142" t="n">
         <v>12806</v>
       </c>
@@ -9638,7 +9920,9 @@
       <c r="G143" t="n">
         <v>0</v>
       </c>
-      <c r="H143" t="inlineStr"/>
+      <c r="H143" t="n">
+        <v>142</v>
+      </c>
       <c r="I143" t="n">
         <v>12638</v>
       </c>
@@ -9710,7 +9994,9 @@
       <c r="G144" t="n">
         <v>0</v>
       </c>
-      <c r="H144" t="inlineStr"/>
+      <c r="H144" t="n">
+        <v>143</v>
+      </c>
       <c r="I144" t="n">
         <v>12568</v>
       </c>
@@ -9776,7 +10062,9 @@
       <c r="G145" t="n">
         <v>0</v>
       </c>
-      <c r="H145" t="inlineStr"/>
+      <c r="H145" t="n">
+        <v>144</v>
+      </c>
       <c r="I145" t="n">
         <v>12627</v>
       </c>
@@ -9842,7 +10130,9 @@
       <c r="G146" t="n">
         <v>0</v>
       </c>
-      <c r="H146" t="inlineStr"/>
+      <c r="H146" t="n">
+        <v>145</v>
+      </c>
       <c r="I146" t="n">
         <v>12146</v>
       </c>
@@ -9908,7 +10198,9 @@
       <c r="G147" t="n">
         <v>0</v>
       </c>
-      <c r="H147" t="inlineStr"/>
+      <c r="H147" t="n">
+        <v>146</v>
+      </c>
       <c r="I147" t="n">
         <v>12400</v>
       </c>
@@ -9980,7 +10272,9 @@
       <c r="G148" t="n">
         <v>0</v>
       </c>
-      <c r="H148" t="inlineStr"/>
+      <c r="H148" t="n">
+        <v>147</v>
+      </c>
       <c r="I148" t="n">
         <v>12288</v>
       </c>
@@ -10052,7 +10346,9 @@
       <c r="G149" t="n">
         <v>0</v>
       </c>
-      <c r="H149" t="inlineStr"/>
+      <c r="H149" t="n">
+        <v>148</v>
+      </c>
       <c r="I149" t="inlineStr"/>
       <c r="J149" t="inlineStr">
         <is>
@@ -10116,7 +10412,9 @@
       <c r="G150" t="n">
         <v>0</v>
       </c>
-      <c r="H150" t="inlineStr"/>
+      <c r="H150" t="n">
+        <v>149</v>
+      </c>
       <c r="I150" t="inlineStr"/>
       <c r="J150" t="inlineStr">
         <is>
@@ -10180,7 +10478,9 @@
       <c r="G151" t="n">
         <v>0</v>
       </c>
-      <c r="H151" t="inlineStr"/>
+      <c r="H151" t="n">
+        <v>150</v>
+      </c>
       <c r="I151" t="inlineStr"/>
       <c r="J151" t="inlineStr">
         <is>
@@ -10244,7 +10544,9 @@
       <c r="G152" t="n">
         <v>0</v>
       </c>
-      <c r="H152" t="inlineStr"/>
+      <c r="H152" t="n">
+        <v>151</v>
+      </c>
       <c r="I152" t="inlineStr"/>
       <c r="J152" t="inlineStr">
         <is>
@@ -10308,7 +10610,9 @@
       <c r="G153" t="n">
         <v>0</v>
       </c>
-      <c r="H153" t="inlineStr"/>
+      <c r="H153" t="n">
+        <v>152</v>
+      </c>
       <c r="I153" t="inlineStr"/>
       <c r="J153" t="inlineStr">
         <is>
@@ -10372,7 +10676,9 @@
       <c r="G154" t="n">
         <v>0</v>
       </c>
-      <c r="H154" t="inlineStr"/>
+      <c r="H154" t="n">
+        <v>153</v>
+      </c>
       <c r="I154" t="inlineStr"/>
       <c r="J154" t="inlineStr">
         <is>
@@ -10436,7 +10742,9 @@
       <c r="G155" t="n">
         <v>0</v>
       </c>
-      <c r="H155" t="inlineStr"/>
+      <c r="H155" t="n">
+        <v>154</v>
+      </c>
       <c r="I155" t="inlineStr"/>
       <c r="J155" t="inlineStr">
         <is>
@@ -10500,7 +10808,9 @@
       <c r="G156" t="n">
         <v>0</v>
       </c>
-      <c r="H156" t="inlineStr"/>
+      <c r="H156" t="n">
+        <v>155</v>
+      </c>
       <c r="I156" t="inlineStr"/>
       <c r="J156" t="inlineStr">
         <is>
@@ -10564,7 +10874,9 @@
       <c r="G157" t="n">
         <v>0</v>
       </c>
-      <c r="H157" t="inlineStr"/>
+      <c r="H157" t="n">
+        <v>156</v>
+      </c>
       <c r="I157" t="inlineStr"/>
       <c r="J157" t="inlineStr">
         <is>
@@ -10628,7 +10940,9 @@
       <c r="G158" t="n">
         <v>0</v>
       </c>
-      <c r="H158" t="inlineStr"/>
+      <c r="H158" t="n">
+        <v>157</v>
+      </c>
       <c r="I158" t="inlineStr"/>
       <c r="J158" t="inlineStr">
         <is>
@@ -10692,7 +11006,9 @@
       <c r="G159" t="n">
         <v>0</v>
       </c>
-      <c r="H159" t="inlineStr"/>
+      <c r="H159" t="n">
+        <v>158</v>
+      </c>
       <c r="I159" t="inlineStr"/>
       <c r="J159" t="inlineStr">
         <is>
@@ -10756,7 +11072,9 @@
       <c r="G160" t="n">
         <v>0</v>
       </c>
-      <c r="H160" t="inlineStr"/>
+      <c r="H160" t="n">
+        <v>159</v>
+      </c>
       <c r="I160" t="inlineStr"/>
       <c r="J160" t="inlineStr">
         <is>
@@ -10820,7 +11138,9 @@
       <c r="G161" t="n">
         <v>0</v>
       </c>
-      <c r="H161" t="inlineStr"/>
+      <c r="H161" t="n">
+        <v>160</v>
+      </c>
       <c r="I161" t="inlineStr"/>
       <c r="J161" t="inlineStr">
         <is>
@@ -10884,7 +11204,9 @@
       <c r="G162" t="n">
         <v>0</v>
       </c>
-      <c r="H162" t="inlineStr"/>
+      <c r="H162" t="n">
+        <v>161</v>
+      </c>
       <c r="I162" t="inlineStr"/>
       <c r="J162" t="inlineStr">
         <is>
@@ -10948,7 +11270,9 @@
       <c r="G163" t="n">
         <v>0</v>
       </c>
-      <c r="H163" t="inlineStr"/>
+      <c r="H163" t="n">
+        <v>162</v>
+      </c>
       <c r="I163" t="inlineStr"/>
       <c r="J163" t="inlineStr">
         <is>
@@ -11012,7 +11336,9 @@
       <c r="G164" t="n">
         <v>0</v>
       </c>
-      <c r="H164" t="inlineStr"/>
+      <c r="H164" t="n">
+        <v>163</v>
+      </c>
       <c r="I164" t="inlineStr"/>
       <c r="J164" t="inlineStr">
         <is>
@@ -11076,7 +11402,9 @@
       <c r="G165" t="n">
         <v>0</v>
       </c>
-      <c r="H165" t="inlineStr"/>
+      <c r="H165" t="n">
+        <v>164</v>
+      </c>
       <c r="I165" t="inlineStr"/>
       <c r="J165" t="inlineStr">
         <is>
@@ -11140,7 +11468,9 @@
       <c r="G166" t="n">
         <v>0</v>
       </c>
-      <c r="H166" t="inlineStr"/>
+      <c r="H166" t="n">
+        <v>165</v>
+      </c>
       <c r="I166" t="inlineStr"/>
       <c r="J166" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
update data package at: 2026-08-31T10:18:24
</commit_message>
<xml_diff>
--- a/data/BASE_DETALHAMENTO_OBRAS.xlsx
+++ b/data/BASE_DETALHAMENTO_OBRAS.xlsx
@@ -499,42 +499,42 @@
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>VALOR TESOURO 2026 (R$)</t>
+          <t>VALOR TESOURO 2027 (R$)</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>VALOR OUTROS 2026 (R$)</t>
+          <t>VALOR OUTROS 2027 (R$)</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>VALOR TESOURO 2027 (R$)</t>
+          <t>VALOR TESOURO 2028 (R$)</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>VALOR OUTROS 2027 (R$)</t>
+          <t>VALOR OUTROS 2028 (R$)</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>VALOR TESOURO 2028 (R$)</t>
+          <t>VALOR TESOURO 2029 (R$)</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>VALOR OUTROS 2028 (R$)</t>
+          <t>VALOR OUTROS 2029 (R$)</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>VALOR TESOURO 2029 (R$)</t>
+          <t>VALOR TESOURO 2030 (R$)</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>VALOR OUTROS 2029 (R$)</t>
+          <t>VALOR OUTROS 2030 (R$)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update data package at: 2026-09-09T07:14:01
</commit_message>
<xml_diff>
--- a/data/BASE_DETALHAMENTO_OBRAS.xlsx
+++ b/data/BASE_DETALHAMENTO_OBRAS.xlsx
@@ -842,7 +842,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -916,7 +916,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -990,7 +990,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -8440,7 +8440,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M118" t="n">
@@ -8597,7 +8597,7 @@
         <v>150000</v>
       </c>
       <c r="R120" t="n">
-        <v>20000000</v>
+        <v>19850000</v>
       </c>
       <c r="S120" t="inlineStr"/>
       <c r="T120" t="inlineStr"/>
@@ -8914,7 +8914,7 @@
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M125" t="n">
@@ -8986,7 +8986,7 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M126" t="n">
@@ -16982,7 +16982,7 @@
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>METRO QUADRADO</t>
+          <t>130</t>
         </is>
       </c>
       <c r="M247" t="n">
@@ -17826,7 +17826,7 @@
       </c>
       <c r="L260" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M260" t="n">
@@ -17900,7 +17900,7 @@
       </c>
       <c r="L261" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M261" t="n">
@@ -17974,7 +17974,7 @@
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M262" t="n">
@@ -18048,7 +18048,7 @@
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M263" t="n">
@@ -18122,7 +18122,7 @@
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M264" t="n">
@@ -18196,7 +18196,7 @@
       </c>
       <c r="L265" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M265" t="n">
@@ -18270,7 +18270,7 @@
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M266" t="n">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="L267" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M267" t="n">
@@ -18418,7 +18418,7 @@
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M268" t="n">
@@ -18492,7 +18492,7 @@
       </c>
       <c r="L269" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M269" t="n">
@@ -18566,7 +18566,7 @@
       </c>
       <c r="L270" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M270" t="n">
@@ -18640,7 +18640,7 @@
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M271" t="n">
@@ -18714,7 +18714,7 @@
       </c>
       <c r="L272" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M272" t="n">
@@ -18788,7 +18788,7 @@
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M273" t="n">
@@ -18862,7 +18862,7 @@
       </c>
       <c r="L274" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M274" t="n">
@@ -18934,7 +18934,7 @@
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M275" t="n">
@@ -19006,7 +19006,7 @@
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M276" t="n">
@@ -19078,7 +19078,7 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M277" t="n">
@@ -19150,7 +19150,7 @@
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M278" t="n">
@@ -19224,7 +19224,7 @@
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M279" t="n">
@@ -19298,7 +19298,7 @@
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M280" t="n">
@@ -19372,7 +19372,7 @@
       </c>
       <c r="L281" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M281" t="n">
@@ -19444,7 +19444,7 @@
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>UNIDADE</t>
+          <t>207</t>
         </is>
       </c>
       <c r="M282" t="n">

</xml_diff>

<commit_message>
update data package at: 2026-09-09T07:16:37
</commit_message>
<xml_diff>
--- a/data/BASE_DETALHAMENTO_OBRAS.xlsx
+++ b/data/BASE_DETALHAMENTO_OBRAS.xlsx
@@ -842,7 +842,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -916,7 +916,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -990,7 +990,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -1064,7 +1064,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -8440,7 +8440,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M118" t="n">
@@ -8914,7 +8914,7 @@
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M125" t="n">
@@ -8986,7 +8986,7 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M126" t="n">
@@ -16982,7 +16982,7 @@
       </c>
       <c r="L247" t="inlineStr">
         <is>
-          <t>130</t>
+          <t>METRO QUADRADO</t>
         </is>
       </c>
       <c r="M247" t="n">
@@ -17826,7 +17826,7 @@
       </c>
       <c r="L260" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M260" t="n">
@@ -17900,7 +17900,7 @@
       </c>
       <c r="L261" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M261" t="n">
@@ -17974,7 +17974,7 @@
       </c>
       <c r="L262" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M262" t="n">
@@ -18048,7 +18048,7 @@
       </c>
       <c r="L263" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M263" t="n">
@@ -18122,7 +18122,7 @@
       </c>
       <c r="L264" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M264" t="n">
@@ -18196,7 +18196,7 @@
       </c>
       <c r="L265" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M265" t="n">
@@ -18270,7 +18270,7 @@
       </c>
       <c r="L266" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M266" t="n">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="L267" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M267" t="n">
@@ -18418,7 +18418,7 @@
       </c>
       <c r="L268" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M268" t="n">
@@ -18492,7 +18492,7 @@
       </c>
       <c r="L269" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M269" t="n">
@@ -18566,7 +18566,7 @@
       </c>
       <c r="L270" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M270" t="n">
@@ -18640,7 +18640,7 @@
       </c>
       <c r="L271" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M271" t="n">
@@ -18714,7 +18714,7 @@
       </c>
       <c r="L272" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M272" t="n">
@@ -18788,7 +18788,7 @@
       </c>
       <c r="L273" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M273" t="n">
@@ -18862,7 +18862,7 @@
       </c>
       <c r="L274" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M274" t="n">
@@ -18934,7 +18934,7 @@
       </c>
       <c r="L275" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M275" t="n">
@@ -19006,7 +19006,7 @@
       </c>
       <c r="L276" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M276" t="n">
@@ -19078,7 +19078,7 @@
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M277" t="n">
@@ -19150,7 +19150,7 @@
       </c>
       <c r="L278" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M278" t="n">
@@ -19224,7 +19224,7 @@
       </c>
       <c r="L279" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M279" t="n">
@@ -19298,7 +19298,7 @@
       </c>
       <c r="L280" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M280" t="n">
@@ -19372,7 +19372,7 @@
       </c>
       <c r="L281" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M281" t="n">
@@ -19444,7 +19444,7 @@
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>UNIDADE</t>
         </is>
       </c>
       <c r="M282" t="n">

</xml_diff>

<commit_message>
update data package at: 2026-09-09T12:29:06
</commit_message>
<xml_diff>
--- a/data/BASE_DETALHAMENTO_OBRAS.xlsx
+++ b/data/BASE_DETALHAMENTO_OBRAS.xlsx
@@ -8034,7 +8034,7 @@
       <c r="I112" t="inlineStr"/>
       <c r="J112" t="inlineStr">
         <is>
-          <t>REDIMENSIONAMENTO DE REDE ELÉTRICA (NRPMSO'S) - Garantir a segurança elétrica para implementação de novos equipamentos</t>
+          <t>REDIMENSIONAMENTO DE REDE ELÉTRICA (NRPMSO`S) - Garantir a segurança elétrica para implementação de novos equipamentos</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -15916,7 +15916,7 @@
       <c r="I231" t="inlineStr"/>
       <c r="J231" t="inlineStr">
         <is>
-          <t>CONSERVAÇÃO DA MALHA VIÁRIA DAS 40ª URG'S</t>
+          <t>CONSERVAÇÃO DA MALHA VIÁRIA DAS 40ª URG`S</t>
         </is>
       </c>
       <c r="K231" t="inlineStr">

</xml_diff>